<commit_message>
Feb 7 2024 TMTT0038660 std snd Super user
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeRecordManagerForFVAStandardUserOntheSFLightningView.xlsx
+++ b/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeRecordManagerForFVAStandardUserOntheSFLightningView.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE8B288-4709-4F2A-8CA7-2E7CE74BCC49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FBF6DD-FC14-41AF-AEF6-B00A9FF31B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="44">
   <si>
     <t>Global Search User</t>
   </si>
@@ -164,6 +164,18 @@
   </si>
   <si>
     <t>6</t>
+  </si>
+  <si>
+    <t>GroupName</t>
+  </si>
+  <si>
+    <t>Time Tracking PV</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>CF Financial User</t>
   </si>
 </sst>
 </file>
@@ -500,21 +512,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>